<commit_message>
Added readme and psychometric sctucture script
</commit_message>
<xml_diff>
--- a/results/tables/table-summaries.xlsx
+++ b/results/tables/table-summaries.xlsx
@@ -26,13 +26,14 @@
     <sheet name="Table S18" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="Table S19" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="Table S20" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Table S22" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Table S21" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Table S22" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="649" uniqueCount="649">
   <si>
     <t xml:space="preserve">V1</t>
   </si>
@@ -1075,6 +1076,843 @@
     <t xml:space="preserve">0.3</t>
   </si>
   <si>
+    <t xml:space="preserve">3.44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.25 - 3.62</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35.52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.26 - 0.27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.972</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.1 - 0.43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.219</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.13 - 0.42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.294</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.23 - 0.31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.04 - 0.49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.67</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.096</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.03 - 0.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.23 - 0.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.777</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.14 - 0.39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.358</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.02 - 0.51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.82</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.08 - 0.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.18 - 0.36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.517</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.54 - 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.93</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.053</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.82 - -0.27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-3.82</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.81 - -0.31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.35 - -0.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-11.87</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.08 - 0.02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.189</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus2:categoryNon Artists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.29 - 0.48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.622</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus3:categoryNon Artists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.43 - 0.32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.774</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus4:categoryNon Artists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.45 - 0.32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.753</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus5:categoryNon Artists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.41 - 0.38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.94</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus6:categoryNon Artists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.58 - 0.17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.293</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus7:categoryNon Artists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.67 - 0.08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.121</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus8:categoryNon Artists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.43 - 0.33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.798</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus9:categoryNon Artists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.55 - 0.21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.89</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.374</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus10:categoryNon Artists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.49 - 0.28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.595</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus11:categoryNon Artists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.46 - 0.29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus12:categoryNon Artists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.44 - 0.32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.769</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus2:categoryHuman Inspired GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.25 - 0.54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.71</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.475</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus3:categoryHuman Inspired GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.73 - 0.14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.186</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus4:categoryHuman Inspired GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.35 - 0.39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.931</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus5:categoryHuman Inspired GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.11 - 0.86</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus6:categoryHuman Inspired GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.47 - 0.29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.632</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus7:categoryHuman Inspired GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.22 - 0.56</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.84</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus8:categoryHuman Inspired GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.1 - 0.66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.145</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus9:categoryHuman Inspired GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.18 - 0.61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus11:categoryHuman Inspired GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.24 - 0.55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.78</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.437</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus12:categoryHuman Inspired GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.5 - 0.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.993</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus2:categorySelf-Guided GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.48 - 0.24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.512</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus3:categorySelf-Guided GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.73 - 0.02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.88</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.061</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus4:categorySelf-Guided GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.6 - 0.16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.266</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus5:categorySelf-Guided GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.59 - 0.18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.295</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus6:categorySelf-Guided GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.73 - 0.05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.72</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.086</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus7:categorySelf-Guided GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.77 - -0.02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-2.04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus8:categorySelf-Guided GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.78 - -0.02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-2.08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.038</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus9:categorySelf-Guided GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.65 - 0.09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.144</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus11:categorySelf-Guided GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.84 - -0.09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-2.42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus12:categorySelf-Guided GenAI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.52 - 0.21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus2:raterTypeGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.2 - -0.08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-4.43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus3:raterTypeGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.03 - 0.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.98</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.329</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus4:raterTypeGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.03 - 0.16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus5:raterTypeGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.3 - -0.18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-7.38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus6:raterTypeGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.23 - -0.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-5.35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus7:raterTypeGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.06 - 0.06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.987</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus8:raterTypeGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.04 - 0.08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.534</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus9:raterTypeGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.31 - -0.18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-7.61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus10:raterTypeGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.04 - 0.12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.302</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus11:raterTypeGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.02 - 0.15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus12:raterTypeGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.12 - 0.01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.101</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus2:raterTypeGuidedGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.02 - 0.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus3:raterTypeGuidedGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1 - 0.23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus4:raterTypeGuidedGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1 - 0.22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus5:raterTypeGuidedGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.02 - 0.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.161</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus6:raterTypeGuidedGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.04 - 0.09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.477</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus7:raterTypeGuidedGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.08 - 0.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus8:raterTypeGuidedGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.08 - 0.21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus9:raterTypeGuidedGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.05 - 0.08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.705</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus10:raterTypeGuidedGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.05 - 0.21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus11:raterTypeGuidedGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.12 - 0.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.71</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stimulus12:raterTypeGuidedGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.06 - 0.07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.985</t>
+  </si>
+  <si>
+    <t xml:space="preserve">categoryNon Artists:raterTypeGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.3 - 0.37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18.39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">categoryHuman Inspired GenAI:raterTypeGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.5 - 0.58</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27.68</t>
+  </si>
+  <si>
+    <t xml:space="preserve">categorySelf-Guided GenAI:raterTypeGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.58 - 0.65</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31.51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">categoryNon Artists:raterTypeGuidedGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.08 - 0.15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">categoryHuman Inspired GenAI:raterTypeGuidedGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-6.95</t>
+  </si>
+  <si>
+    <t xml:space="preserve">categorySelf-Guided GenAI:raterTypeGuidedGPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.29 - -0.21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-12.63</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.203</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.31</t>
+  </si>
+  <si>
     <t xml:space="preserve">3.87</t>
   </si>
   <si>
@@ -1139,12 +1977,6 @@
   </si>
   <si>
     <t xml:space="preserve">1.08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.145</t>
   </si>
   <si>
     <t xml:space="preserve">0.381</t>
@@ -5987,7 +6819,7 @@
         <v>347</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>111</v>
       </c>
       <c r="D5" t="s">
         <v>348</v>
@@ -6004,16 +6836,1787 @@
         <v>350</v>
       </c>
       <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="s">
         <v>351</v>
+      </c>
+      <c r="E6" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>353</v>
+      </c>
+      <c r="B7" t="s">
+        <v>354</v>
+      </c>
+      <c r="C7" t="s">
+        <v>276</v>
+      </c>
+      <c r="D7" t="s">
+        <v>355</v>
+      </c>
+      <c r="E7" t="s">
+        <v>356</v>
+      </c>
+      <c r="F7" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>358</v>
+      </c>
+      <c r="B8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" t="s">
+        <v>359</v>
+      </c>
+      <c r="E8" t="s">
+        <v>360</v>
+      </c>
+      <c r="F8" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>362</v>
+      </c>
+      <c r="B9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" t="s">
+        <v>363</v>
+      </c>
+      <c r="E9" t="s">
+        <v>364</v>
+      </c>
+      <c r="F9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>365</v>
+      </c>
+      <c r="B10" t="s">
+        <v>366</v>
+      </c>
+      <c r="C10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" t="s">
+        <v>367</v>
+      </c>
+      <c r="E10" t="s">
+        <v>368</v>
+      </c>
+      <c r="F10" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>370</v>
+      </c>
+      <c r="B11" t="s">
+        <v>371</v>
+      </c>
+      <c r="C11" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" t="s">
+        <v>372</v>
+      </c>
+      <c r="E11" t="s">
+        <v>373</v>
+      </c>
+      <c r="F11" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>374</v>
+      </c>
+      <c r="B12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" t="s">
+        <v>375</v>
+      </c>
+      <c r="E12" t="s">
+        <v>364</v>
+      </c>
+      <c r="F12" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>377</v>
+      </c>
+      <c r="B13" t="s">
+        <v>97</v>
+      </c>
+      <c r="C13" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" t="s">
+        <v>378</v>
+      </c>
+      <c r="E13" t="s">
+        <v>379</v>
+      </c>
+      <c r="F13" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>381</v>
+      </c>
+      <c r="B14" t="s">
+        <v>371</v>
+      </c>
+      <c r="C14" t="s">
+        <v>276</v>
+      </c>
+      <c r="D14" t="s">
+        <v>382</v>
+      </c>
+      <c r="E14" t="s">
+        <v>383</v>
+      </c>
+      <c r="F14" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>384</v>
+      </c>
+      <c r="B15" t="s">
+        <v>324</v>
+      </c>
+      <c r="C15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" t="s">
+        <v>385</v>
+      </c>
+      <c r="E15" t="s">
+        <v>386</v>
+      </c>
+      <c r="F15" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>388</v>
+      </c>
+      <c r="B16" t="s">
+        <v>345</v>
+      </c>
+      <c r="C16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" t="s">
+        <v>389</v>
+      </c>
+      <c r="E16" t="s">
+        <v>231</v>
+      </c>
+      <c r="F16" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>314</v>
+      </c>
+      <c r="B17" t="s">
+        <v>211</v>
+      </c>
+      <c r="C17" t="s">
+        <v>35</v>
+      </c>
+      <c r="D17" t="s">
+        <v>391</v>
+      </c>
+      <c r="E17" t="s">
+        <v>392</v>
+      </c>
+      <c r="F17" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>317</v>
+      </c>
+      <c r="B18" t="s">
+        <v>394</v>
+      </c>
+      <c r="C18" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" t="s">
+        <v>395</v>
+      </c>
+      <c r="E18" t="s">
+        <v>396</v>
+      </c>
+      <c r="F18" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>320</v>
+      </c>
+      <c r="B19" t="s">
+        <v>145</v>
+      </c>
+      <c r="C19" t="s">
+        <v>276</v>
+      </c>
+      <c r="D19" t="s">
+        <v>397</v>
+      </c>
+      <c r="E19" t="s">
+        <v>398</v>
+      </c>
+      <c r="F19" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>308</v>
+      </c>
+      <c r="B20" t="s">
+        <v>265</v>
+      </c>
+      <c r="C20" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" t="s">
+        <v>399</v>
+      </c>
+      <c r="E20" t="s">
+        <v>400</v>
+      </c>
+      <c r="F20" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>311</v>
+      </c>
+      <c r="B21" t="s">
+        <v>401</v>
+      </c>
+      <c r="C21" t="s">
+        <v>22</v>
+      </c>
+      <c r="D21" t="s">
+        <v>402</v>
+      </c>
+      <c r="E21" t="s">
+        <v>403</v>
+      </c>
+      <c r="F21" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>405</v>
+      </c>
+      <c r="B22" t="s">
+        <v>111</v>
+      </c>
+      <c r="C22" t="s">
+        <v>244</v>
+      </c>
+      <c r="D22" t="s">
+        <v>406</v>
+      </c>
+      <c r="E22" t="s">
+        <v>407</v>
+      </c>
+      <c r="F22" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>409</v>
+      </c>
+      <c r="B23" t="s">
+        <v>410</v>
+      </c>
+      <c r="C23" t="s">
+        <v>244</v>
+      </c>
+      <c r="D23" t="s">
+        <v>411</v>
+      </c>
+      <c r="E23" t="s">
+        <v>190</v>
+      </c>
+      <c r="F23" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>413</v>
+      </c>
+      <c r="B24" t="s">
+        <v>410</v>
+      </c>
+      <c r="C24" t="s">
+        <v>414</v>
+      </c>
+      <c r="D24" t="s">
+        <v>415</v>
+      </c>
+      <c r="E24" t="s">
+        <v>416</v>
+      </c>
+      <c r="F24" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>418</v>
+      </c>
+      <c r="B25" t="s">
+        <v>126</v>
+      </c>
+      <c r="C25" t="s">
+        <v>414</v>
+      </c>
+      <c r="D25" t="s">
+        <v>419</v>
+      </c>
+      <c r="E25" t="s">
+        <v>420</v>
+      </c>
+      <c r="F25" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>422</v>
+      </c>
+      <c r="B26" t="s">
+        <v>423</v>
+      </c>
+      <c r="C26" t="s">
+        <v>244</v>
+      </c>
+      <c r="D26" t="s">
+        <v>424</v>
+      </c>
+      <c r="E26" t="s">
+        <v>425</v>
+      </c>
+      <c r="F26" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>427</v>
+      </c>
+      <c r="B27" t="s">
+        <v>190</v>
+      </c>
+      <c r="C27" t="s">
+        <v>244</v>
+      </c>
+      <c r="D27" t="s">
+        <v>428</v>
+      </c>
+      <c r="E27" t="s">
+        <v>429</v>
+      </c>
+      <c r="F27" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>431</v>
+      </c>
+      <c r="B28" t="s">
+        <v>204</v>
+      </c>
+      <c r="C28" t="s">
+        <v>244</v>
+      </c>
+      <c r="D28" t="s">
+        <v>432</v>
+      </c>
+      <c r="E28" t="s">
+        <v>249</v>
+      </c>
+      <c r="F28" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>434</v>
+      </c>
+      <c r="B29" t="s">
+        <v>435</v>
+      </c>
+      <c r="C29" t="s">
+        <v>244</v>
+      </c>
+      <c r="D29" t="s">
+        <v>436</v>
+      </c>
+      <c r="E29" t="s">
+        <v>437</v>
+      </c>
+      <c r="F29" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>439</v>
+      </c>
+      <c r="B30" t="s">
+        <v>440</v>
+      </c>
+      <c r="C30" t="s">
+        <v>414</v>
+      </c>
+      <c r="D30" t="s">
+        <v>441</v>
+      </c>
+      <c r="E30" t="s">
+        <v>442</v>
+      </c>
+      <c r="F30" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>444</v>
+      </c>
+      <c r="B31" t="s">
+        <v>175</v>
+      </c>
+      <c r="C31" t="s">
+        <v>244</v>
+      </c>
+      <c r="D31" t="s">
+        <v>445</v>
+      </c>
+      <c r="E31" t="s">
+        <v>46</v>
+      </c>
+      <c r="F31" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>446</v>
+      </c>
+      <c r="B32" t="s">
+        <v>410</v>
+      </c>
+      <c r="C32" t="s">
+        <v>244</v>
+      </c>
+      <c r="D32" t="s">
+        <v>447</v>
+      </c>
+      <c r="E32" t="s">
+        <v>190</v>
+      </c>
+      <c r="F32" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>449</v>
+      </c>
+      <c r="B33" t="s">
+        <v>35</v>
+      </c>
+      <c r="C33" t="s">
+        <v>414</v>
+      </c>
+      <c r="D33" t="s">
+        <v>450</v>
+      </c>
+      <c r="E33" t="s">
+        <v>451</v>
+      </c>
+      <c r="F33" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>453</v>
+      </c>
+      <c r="B34" t="s">
+        <v>265</v>
+      </c>
+      <c r="C34" t="s">
+        <v>454</v>
+      </c>
+      <c r="D34" t="s">
+        <v>455</v>
+      </c>
+      <c r="E34" t="s">
+        <v>456</v>
+      </c>
+      <c r="F34" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>458</v>
+      </c>
+      <c r="B35" t="s">
+        <v>16</v>
+      </c>
+      <c r="C35" t="s">
+        <v>244</v>
+      </c>
+      <c r="D35" t="s">
+        <v>459</v>
+      </c>
+      <c r="E35" t="s">
+        <v>345</v>
+      </c>
+      <c r="F35" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>461</v>
+      </c>
+      <c r="B36" t="s">
+        <v>242</v>
+      </c>
+      <c r="C36" t="s">
+        <v>244</v>
+      </c>
+      <c r="D36" t="s">
+        <v>462</v>
+      </c>
+      <c r="E36" t="s">
+        <v>463</v>
+      </c>
+      <c r="F36" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>464</v>
+      </c>
+      <c r="B37" t="s">
+        <v>465</v>
+      </c>
+      <c r="C37" t="s">
+        <v>244</v>
+      </c>
+      <c r="D37" t="s">
+        <v>466</v>
+      </c>
+      <c r="E37" t="s">
+        <v>163</v>
+      </c>
+      <c r="F37" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>468</v>
+      </c>
+      <c r="B38" t="s">
+        <v>82</v>
+      </c>
+      <c r="C38" t="s">
+        <v>414</v>
+      </c>
+      <c r="D38" t="s">
+        <v>469</v>
+      </c>
+      <c r="E38" t="s">
+        <v>470</v>
+      </c>
+      <c r="F38" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>472</v>
+      </c>
+      <c r="B39" t="s">
+        <v>364</v>
+      </c>
+      <c r="C39" t="s">
+        <v>244</v>
+      </c>
+      <c r="D39" t="s">
+        <v>473</v>
+      </c>
+      <c r="E39" t="s">
+        <v>474</v>
+      </c>
+      <c r="F39" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>476</v>
+      </c>
+      <c r="B40" t="s">
+        <v>222</v>
+      </c>
+      <c r="C40" t="s">
+        <v>414</v>
+      </c>
+      <c r="D40" t="s">
+        <v>477</v>
+      </c>
+      <c r="E40" t="s">
+        <v>478</v>
+      </c>
+      <c r="F40" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>479</v>
+      </c>
+      <c r="B41" t="s">
+        <v>354</v>
+      </c>
+      <c r="C41" t="s">
+        <v>414</v>
+      </c>
+      <c r="D41" t="s">
+        <v>480</v>
+      </c>
+      <c r="E41" t="s">
+        <v>481</v>
+      </c>
+      <c r="F41" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>483</v>
+      </c>
+      <c r="B42" t="s">
+        <v>19</v>
+      </c>
+      <c r="C42" t="s">
+        <v>484</v>
+      </c>
+      <c r="D42" t="s">
+        <v>485</v>
+      </c>
+      <c r="E42" t="s">
+        <v>126</v>
+      </c>
+      <c r="F42" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>487</v>
+      </c>
+      <c r="B43" t="s">
+        <v>488</v>
+      </c>
+      <c r="C43" t="s">
+        <v>153</v>
+      </c>
+      <c r="D43" t="s">
+        <v>489</v>
+      </c>
+      <c r="E43" t="s">
+        <v>490</v>
+      </c>
+      <c r="F43" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>492</v>
+      </c>
+      <c r="B44" t="s">
+        <v>101</v>
+      </c>
+      <c r="C44" t="s">
+        <v>244</v>
+      </c>
+      <c r="D44" t="s">
+        <v>493</v>
+      </c>
+      <c r="E44" t="s">
+        <v>494</v>
+      </c>
+      <c r="F44" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>496</v>
+      </c>
+      <c r="B45" t="s">
+        <v>133</v>
+      </c>
+      <c r="C45" t="s">
+        <v>244</v>
+      </c>
+      <c r="D45" t="s">
+        <v>497</v>
+      </c>
+      <c r="E45" t="s">
+        <v>498</v>
+      </c>
+      <c r="F45" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>500</v>
+      </c>
+      <c r="B46" t="s">
+        <v>501</v>
+      </c>
+      <c r="C46" t="s">
+        <v>414</v>
+      </c>
+      <c r="D46" t="s">
+        <v>502</v>
+      </c>
+      <c r="E46" t="s">
+        <v>425</v>
+      </c>
+      <c r="F46" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>504</v>
+      </c>
+      <c r="B47" t="s">
+        <v>505</v>
+      </c>
+      <c r="C47" t="s">
+        <v>414</v>
+      </c>
+      <c r="D47" t="s">
+        <v>506</v>
+      </c>
+      <c r="E47" t="s">
+        <v>507</v>
+      </c>
+      <c r="F47" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>509</v>
+      </c>
+      <c r="B48" t="s">
+        <v>510</v>
+      </c>
+      <c r="C48" t="s">
+        <v>244</v>
+      </c>
+      <c r="D48" t="s">
+        <v>511</v>
+      </c>
+      <c r="E48" t="s">
+        <v>512</v>
+      </c>
+      <c r="F48" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>513</v>
+      </c>
+      <c r="B49" t="s">
+        <v>514</v>
+      </c>
+      <c r="C49" t="s">
+        <v>244</v>
+      </c>
+      <c r="D49" t="s">
+        <v>515</v>
+      </c>
+      <c r="E49" t="s">
+        <v>516</v>
+      </c>
+      <c r="F49" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>518</v>
+      </c>
+      <c r="B50" t="s">
+        <v>128</v>
+      </c>
+      <c r="C50" t="s">
+        <v>244</v>
+      </c>
+      <c r="D50" t="s">
+        <v>519</v>
+      </c>
+      <c r="E50" t="s">
+        <v>520</v>
+      </c>
+      <c r="F50" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>522</v>
+      </c>
+      <c r="B51" t="s">
+        <v>523</v>
+      </c>
+      <c r="C51" t="s">
+        <v>244</v>
+      </c>
+      <c r="D51" t="s">
+        <v>524</v>
+      </c>
+      <c r="E51" t="s">
+        <v>525</v>
+      </c>
+      <c r="F51" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>527</v>
+      </c>
+      <c r="B52" t="s">
+        <v>528</v>
+      </c>
+      <c r="C52" t="s">
+        <v>244</v>
+      </c>
+      <c r="D52" t="s">
+        <v>529</v>
+      </c>
+      <c r="E52" t="s">
+        <v>50</v>
+      </c>
+      <c r="F52" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s">
+        <v>531</v>
+      </c>
+      <c r="B53" t="s">
+        <v>220</v>
+      </c>
+      <c r="C53" t="s">
+        <v>22</v>
+      </c>
+      <c r="D53" t="s">
+        <v>532</v>
+      </c>
+      <c r="E53" t="s">
+        <v>533</v>
+      </c>
+      <c r="F53" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>534</v>
+      </c>
+      <c r="B54" t="s">
+        <v>22</v>
+      </c>
+      <c r="C54" t="s">
+        <v>22</v>
+      </c>
+      <c r="D54" t="s">
+        <v>535</v>
+      </c>
+      <c r="E54" t="s">
+        <v>536</v>
+      </c>
+      <c r="F54" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s">
+        <v>538</v>
+      </c>
+      <c r="B55" t="s">
+        <v>345</v>
+      </c>
+      <c r="C55" t="s">
+        <v>22</v>
+      </c>
+      <c r="D55" t="s">
+        <v>539</v>
+      </c>
+      <c r="E55" t="s">
+        <v>540</v>
+      </c>
+      <c r="F55" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>542</v>
+      </c>
+      <c r="B56" t="s">
+        <v>279</v>
+      </c>
+      <c r="C56" t="s">
+        <v>22</v>
+      </c>
+      <c r="D56" t="s">
+        <v>543</v>
+      </c>
+      <c r="E56" t="s">
+        <v>544</v>
+      </c>
+      <c r="F56" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>545</v>
+      </c>
+      <c r="B57" t="s">
+        <v>435</v>
+      </c>
+      <c r="C57" t="s">
+        <v>22</v>
+      </c>
+      <c r="D57" t="s">
+        <v>546</v>
+      </c>
+      <c r="E57" t="s">
+        <v>547</v>
+      </c>
+      <c r="F57" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>548</v>
+      </c>
+      <c r="B58" t="s">
+        <v>19</v>
+      </c>
+      <c r="C58" t="s">
+        <v>22</v>
+      </c>
+      <c r="D58" t="s">
+        <v>549</v>
+      </c>
+      <c r="E58" t="s">
+        <v>188</v>
+      </c>
+      <c r="F58" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s">
+        <v>551</v>
+      </c>
+      <c r="B59" t="s">
+        <v>16</v>
+      </c>
+      <c r="C59" t="s">
+        <v>22</v>
+      </c>
+      <c r="D59" t="s">
+        <v>552</v>
+      </c>
+      <c r="E59" t="s">
+        <v>168</v>
+      </c>
+      <c r="F59" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>554</v>
+      </c>
+      <c r="B60" t="s">
+        <v>555</v>
+      </c>
+      <c r="C60" t="s">
+        <v>22</v>
+      </c>
+      <c r="D60" t="s">
+        <v>556</v>
+      </c>
+      <c r="E60" t="s">
+        <v>557</v>
+      </c>
+      <c r="F60" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>558</v>
+      </c>
+      <c r="B61" t="s">
+        <v>42</v>
+      </c>
+      <c r="C61" t="s">
+        <v>42</v>
+      </c>
+      <c r="D61" t="s">
+        <v>559</v>
+      </c>
+      <c r="E61" t="s">
+        <v>560</v>
+      </c>
+      <c r="F61" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
+        <v>562</v>
+      </c>
+      <c r="B62" t="s">
+        <v>159</v>
+      </c>
+      <c r="C62" t="s">
+        <v>22</v>
+      </c>
+      <c r="D62" t="s">
+        <v>563</v>
+      </c>
+      <c r="E62" t="s">
+        <v>564</v>
+      </c>
+      <c r="F62" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
+        <v>566</v>
+      </c>
+      <c r="B63" t="s">
+        <v>204</v>
+      </c>
+      <c r="C63" t="s">
+        <v>22</v>
+      </c>
+      <c r="D63" t="s">
+        <v>567</v>
+      </c>
+      <c r="E63" t="s">
+        <v>568</v>
+      </c>
+      <c r="F63" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>570</v>
+      </c>
+      <c r="B64" t="s">
+        <v>42</v>
+      </c>
+      <c r="C64" t="s">
+        <v>22</v>
+      </c>
+      <c r="D64" t="s">
+        <v>571</v>
+      </c>
+      <c r="E64" t="s">
+        <v>572</v>
+      </c>
+      <c r="F64" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s">
+        <v>573</v>
+      </c>
+      <c r="B65" t="s">
+        <v>82</v>
+      </c>
+      <c r="C65" t="s">
+        <v>22</v>
+      </c>
+      <c r="D65" t="s">
+        <v>574</v>
+      </c>
+      <c r="E65" t="s">
+        <v>575</v>
+      </c>
+      <c r="F65" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>576</v>
+      </c>
+      <c r="B66" t="s">
+        <v>354</v>
+      </c>
+      <c r="C66" t="s">
+        <v>22</v>
+      </c>
+      <c r="D66" t="s">
+        <v>577</v>
+      </c>
+      <c r="E66" t="s">
+        <v>578</v>
+      </c>
+      <c r="F66" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>579</v>
+      </c>
+      <c r="B67" t="s">
+        <v>55</v>
+      </c>
+      <c r="C67" t="s">
+        <v>22</v>
+      </c>
+      <c r="D67" t="s">
+        <v>580</v>
+      </c>
+      <c r="E67" t="s">
+        <v>581</v>
+      </c>
+      <c r="F67" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>583</v>
+      </c>
+      <c r="B68" t="s">
+        <v>16</v>
+      </c>
+      <c r="C68" t="s">
+        <v>22</v>
+      </c>
+      <c r="D68" t="s">
+        <v>584</v>
+      </c>
+      <c r="E68" t="s">
+        <v>451</v>
+      </c>
+      <c r="F68" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>586</v>
+      </c>
+      <c r="B69" t="s">
+        <v>35</v>
+      </c>
+      <c r="C69" t="s">
+        <v>22</v>
+      </c>
+      <c r="D69" t="s">
+        <v>587</v>
+      </c>
+      <c r="E69" t="s">
+        <v>588</v>
+      </c>
+      <c r="F69" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>589</v>
+      </c>
+      <c r="B70" t="s">
+        <v>590</v>
+      </c>
+      <c r="C70" t="s">
+        <v>22</v>
+      </c>
+      <c r="D70" t="s">
+        <v>591</v>
+      </c>
+      <c r="E70" t="s">
+        <v>592</v>
+      </c>
+      <c r="F70" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s">
+        <v>593</v>
+      </c>
+      <c r="B71" t="s">
+        <v>195</v>
+      </c>
+      <c r="C71" t="s">
+        <v>22</v>
+      </c>
+      <c r="D71" t="s">
+        <v>594</v>
+      </c>
+      <c r="E71" t="s">
+        <v>595</v>
+      </c>
+      <c r="F71" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
+        <v>597</v>
+      </c>
+      <c r="B72" t="s">
+        <v>276</v>
+      </c>
+      <c r="C72" t="s">
+        <v>42</v>
+      </c>
+      <c r="D72" t="s">
+        <v>598</v>
+      </c>
+      <c r="E72" t="s">
+        <v>123</v>
+      </c>
+      <c r="F72" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s">
+        <v>599</v>
+      </c>
+      <c r="B73" t="s">
+        <v>153</v>
+      </c>
+      <c r="C73" t="s">
+        <v>22</v>
+      </c>
+      <c r="D73" t="s">
+        <v>600</v>
+      </c>
+      <c r="E73" t="s">
+        <v>601</v>
+      </c>
+      <c r="F73" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="s">
+        <v>602</v>
+      </c>
+      <c r="B74" t="s">
+        <v>19</v>
+      </c>
+      <c r="C74" t="s">
+        <v>22</v>
+      </c>
+      <c r="D74" t="s">
+        <v>603</v>
+      </c>
+      <c r="E74" t="s">
+        <v>16</v>
+      </c>
+      <c r="F74" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="s">
+        <v>605</v>
+      </c>
+      <c r="B75" t="s">
+        <v>324</v>
+      </c>
+      <c r="C75" t="s">
+        <v>16</v>
+      </c>
+      <c r="D75" t="s">
+        <v>606</v>
+      </c>
+      <c r="E75" t="s">
+        <v>607</v>
+      </c>
+      <c r="F75" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="s">
+        <v>608</v>
+      </c>
+      <c r="B76" t="s">
+        <v>245</v>
+      </c>
+      <c r="C76" t="s">
+        <v>16</v>
+      </c>
+      <c r="D76" t="s">
+        <v>609</v>
+      </c>
+      <c r="E76" t="s">
+        <v>610</v>
+      </c>
+      <c r="F76" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="s">
+        <v>611</v>
+      </c>
+      <c r="B77" t="s">
+        <v>168</v>
+      </c>
+      <c r="C77" t="s">
+        <v>16</v>
+      </c>
+      <c r="D77" t="s">
+        <v>612</v>
+      </c>
+      <c r="E77" t="s">
+        <v>613</v>
+      </c>
+      <c r="F77" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="s">
+        <v>614</v>
+      </c>
+      <c r="B78" t="s">
+        <v>97</v>
+      </c>
+      <c r="C78" t="s">
+        <v>16</v>
+      </c>
+      <c r="D78" t="s">
+        <v>615</v>
+      </c>
+      <c r="E78" t="s">
+        <v>616</v>
+      </c>
+      <c r="F78" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="s">
+        <v>617</v>
+      </c>
+      <c r="B79" t="s">
+        <v>220</v>
+      </c>
+      <c r="C79" t="s">
+        <v>16</v>
+      </c>
+      <c r="D79" t="s">
+        <v>335</v>
+      </c>
+      <c r="E79" t="s">
+        <v>618</v>
+      </c>
+      <c r="F79" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="s">
+        <v>619</v>
+      </c>
+      <c r="B80" t="s">
+        <v>555</v>
+      </c>
+      <c r="C80" t="s">
+        <v>16</v>
+      </c>
+      <c r="D80" t="s">
+        <v>620</v>
+      </c>
+      <c r="E80" t="s">
+        <v>621</v>
+      </c>
+      <c r="F80" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="s">
+        <v>7</v>
+      </c>
+      <c r="B81" t="s">
+        <v>7</v>
+      </c>
+      <c r="C81" t="s">
+        <v>7</v>
+      </c>
+      <c r="D81" t="s">
+        <v>7</v>
+      </c>
+      <c r="E81" t="s">
+        <v>7</v>
+      </c>
+      <c r="F81" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="s">
+        <v>25</v>
+      </c>
+      <c r="B82" t="s">
+        <v>7</v>
+      </c>
+      <c r="C82" t="s">
+        <v>7</v>
+      </c>
+      <c r="D82" t="s">
+        <v>7</v>
+      </c>
+      <c r="E82" t="s">
+        <v>7</v>
+      </c>
+      <c r="F82" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="s">
+        <v>7</v>
+      </c>
+      <c r="B83" t="s">
+        <v>7</v>
+      </c>
+      <c r="C83" t="s">
+        <v>7</v>
+      </c>
+      <c r="D83" t="s">
+        <v>7</v>
+      </c>
+      <c r="E83" t="s">
+        <v>26</v>
+      </c>
+      <c r="F83" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="s">
+        <v>28</v>
+      </c>
+      <c r="B84" t="s">
+        <v>7</v>
+      </c>
+      <c r="C84" t="s">
+        <v>7</v>
+      </c>
+      <c r="D84" t="s">
+        <v>7</v>
+      </c>
+      <c r="E84" t="s">
+        <v>622</v>
+      </c>
+      <c r="F84" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="s">
+        <v>7</v>
+      </c>
+      <c r="B85" t="s">
+        <v>7</v>
+      </c>
+      <c r="C85" t="s">
+        <v>7</v>
+      </c>
+      <c r="D85" t="s">
+        <v>7</v>
+      </c>
+      <c r="E85" t="s">
+        <v>7</v>
+      </c>
+      <c r="F85" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="s">
+        <v>31</v>
+      </c>
+      <c r="B86" t="s">
+        <v>7</v>
+      </c>
+      <c r="C86" t="s">
+        <v>7</v>
+      </c>
+      <c r="D86" t="s">
+        <v>7</v>
+      </c>
+      <c r="E86" t="s">
+        <v>7</v>
+      </c>
+      <c r="F86" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="s">
+        <v>7</v>
+      </c>
+      <c r="B87" t="s">
+        <v>7</v>
+      </c>
+      <c r="C87" t="s">
+        <v>7</v>
+      </c>
+      <c r="D87" t="s">
+        <v>7</v>
+      </c>
+      <c r="E87" t="s">
+        <v>32</v>
+      </c>
+      <c r="F87" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="s">
+        <v>34</v>
+      </c>
+      <c r="B88" t="s">
+        <v>7</v>
+      </c>
+      <c r="C88" t="s">
+        <v>7</v>
+      </c>
+      <c r="D88" t="s">
+        <v>7</v>
+      </c>
+      <c r="E88" t="s">
+        <v>624</v>
+      </c>
+      <c r="F88" t="s">
+        <v>625</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>626</v>
+      </c>
+      <c r="C5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
+        <v>627</v>
+      </c>
+      <c r="E5" t="s">
+        <v>628</v>
+      </c>
+      <c r="F5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>629</v>
+      </c>
+      <c r="B6" t="s">
+        <v>630</v>
       </c>
       <c r="C6" t="s">
         <v>22</v>
       </c>
       <c r="D6" t="s">
-        <v>352</v>
+        <v>631</v>
       </c>
       <c r="E6" t="s">
-        <v>353</v>
+        <v>632</v>
       </c>
       <c r="F6" t="s">
         <v>19</v>
@@ -6033,7 +8636,7 @@
         <v>102</v>
       </c>
       <c r="E7" t="s">
-        <v>354</v>
+        <v>633</v>
       </c>
       <c r="F7" t="s">
         <v>19</v>
@@ -6050,10 +8653,10 @@
         <v>42</v>
       </c>
       <c r="D8" t="s">
-        <v>355</v>
+        <v>634</v>
       </c>
       <c r="E8" t="s">
-        <v>356</v>
+        <v>635</v>
       </c>
       <c r="F8" t="s">
         <v>19</v>
@@ -6064,16 +8667,16 @@
         <v>320</v>
       </c>
       <c r="B9" t="s">
-        <v>357</v>
+        <v>636</v>
       </c>
       <c r="C9" t="s">
         <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>358</v>
+        <v>637</v>
       </c>
       <c r="E9" t="s">
-        <v>359</v>
+        <v>638</v>
       </c>
       <c r="F9" t="s">
         <v>19</v>
@@ -6081,7 +8684,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>360</v>
+        <v>639</v>
       </c>
       <c r="B10" t="s">
         <v>19</v>
@@ -6090,18 +8693,18 @@
         <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>361</v>
+        <v>640</v>
       </c>
       <c r="E10" t="s">
         <v>253</v>
       </c>
       <c r="F10" t="s">
-        <v>362</v>
+        <v>641</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>363</v>
+        <v>642</v>
       </c>
       <c r="B11" t="s">
         <v>19</v>
@@ -6110,18 +8713,18 @@
         <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>364</v>
+        <v>643</v>
       </c>
       <c r="E11" t="s">
         <v>81</v>
       </c>
       <c r="F11" t="s">
-        <v>365</v>
+        <v>644</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>366</v>
+        <v>645</v>
       </c>
       <c r="B12" t="s">
         <v>42</v>
@@ -6130,13 +8733,13 @@
         <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>367</v>
+        <v>646</v>
       </c>
       <c r="E12" t="s">
-        <v>368</v>
+        <v>647</v>
       </c>
       <c r="F12" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
     </row>
     <row r="13">
@@ -6213,10 +8816,10 @@
         <v>7</v>
       </c>
       <c r="E16" t="s">
-        <v>370</v>
+        <v>475</v>
       </c>
       <c r="F16" t="s">
-        <v>371</v>
+        <v>648</v>
       </c>
     </row>
     <row r="17">

</xml_diff>